<commit_message>
excell small sem erros
</commit_message>
<xml_diff>
--- a/static/files/MOCK_DATA_SMALL.xlsx
+++ b/static/files/MOCK_DATA_SMALL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell 2\Desktop\faculdade\3 ano\TFC\CGI-Process-Monitoring-302-303\static\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF50140-BD71-4BE4-A821-8DDC21851D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C684F3C-E583-4687-B109-A390FD96C46D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -665,18 +665,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I21"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.8984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.25" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="10" max="10" width="10.8984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="10.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -693,7 +693,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -706,11 +706,11 @@
       <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="I2">
+      <c r="E2">
         <v>8206365164</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -727,7 +727,7 @@
         <v>1725612465</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -744,7 +744,7 @@
         <v>8162949638</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -761,7 +761,7 @@
         <v>8081690625</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -778,7 +778,7 @@
         <v>4491262936</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -795,7 +795,7 @@
         <v>4254711311</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -812,7 +812,7 @@
         <v>4637704508</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -829,7 +829,7 @@
         <v>2171915720</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -846,7 +846,7 @@
         <v>6975511870</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -863,7 +863,7 @@
         <v>8285272964</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>45</v>
       </c>
@@ -880,7 +880,7 @@
         <v>7986855354</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>49</v>
       </c>
@@ -897,7 +897,7 @@
         <v>1173272278</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>53</v>
       </c>
@@ -914,7 +914,7 @@
         <v>4661283111</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -931,7 +931,7 @@
         <v>5886444948</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>61</v>
       </c>
@@ -948,7 +948,7 @@
         <v>7739529536</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>65</v>
       </c>
@@ -965,7 +965,7 @@
         <v>4675649905</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -982,7 +982,7 @@
         <v>3021677361</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>73</v>
       </c>
@@ -999,7 +999,7 @@
         <v>1724480025</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>77</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>7007063399</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>81</v>
       </c>

</xml_diff>

<commit_message>
API calls every 10 seconds ETL done
</commit_message>
<xml_diff>
--- a/static/files/MOCK_DATA_SMALL.xlsx
+++ b/static/files/MOCK_DATA_SMALL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell 2\Desktop\faculdade\3 ano\TFC\CGI-Process-Monitoring-302-303\static\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C684F3C-E583-4687-B109-A390FD96C46D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6434A9E8-F277-43D1-AD69-FCDD2AB3B2A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -665,7 +665,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.875" bestFit="1" customWidth="1"/>
@@ -676,7 +676,7 @@
     <col min="9" max="10" width="10.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -693,7 +693,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -706,11 +706,11 @@
       <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>8206365164</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -723,11 +723,11 @@
       <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="E3">
+      <c r="G3">
         <v>1725612465</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -744,7 +744,7 @@
         <v>8162949638</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -761,7 +761,7 @@
         <v>8081690625</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -778,7 +778,7 @@
         <v>4491262936</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -795,7 +795,7 @@
         <v>4254711311</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -812,7 +812,7 @@
         <v>4637704508</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -829,7 +829,7 @@
         <v>2171915720</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -846,7 +846,7 @@
         <v>6975511870</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -863,7 +863,7 @@
         <v>8285272964</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>45</v>
       </c>
@@ -880,7 +880,7 @@
         <v>7986855354</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>49</v>
       </c>
@@ -897,7 +897,7 @@
         <v>1173272278</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>53</v>
       </c>
@@ -914,7 +914,7 @@
         <v>4661283111</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -931,7 +931,7 @@
         <v>5886444948</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>61</v>
       </c>

</xml_diff>

<commit_message>
- `services.py Operational_plat` excel to pdf and show only rows with empty fields
</commit_message>
<xml_diff>
--- a/static/files/MOCK_DATA_SMALL.xlsx
+++ b/static/files/MOCK_DATA_SMALL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell 4\Desktop\TFC\CGI-Process-Monitoring-302-303\static\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell 3\PycharmProjects\Project\CGI-Process-Monitoring-302-303\static\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95BC9B08-2CFC-43DA-ABF7-872BF56214E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{822DB8BE-8C89-42C6-BB28-C875240A96A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
   <si>
     <t>first_name</t>
   </si>
@@ -275,9 +275,6 @@
   </si>
   <si>
     <t>55068 Hintze Court</t>
-  </si>
-  <si>
-    <t>x</t>
   </si>
 </sst>
 </file>
@@ -294,6 +291,7 @@
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -716,9 +714,7 @@
       <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" t="s">
-        <v>85</v>
-      </c>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -733,9 +729,7 @@
       <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="F3" t="s">
-        <v>85</v>
-      </c>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">

</xml_diff>

<commit_message>
again the same thing with folder
</commit_message>
<xml_diff>
--- a/static/files/MOCK_DATA_SMALL.xlsx
+++ b/static/files/MOCK_DATA_SMALL.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26501"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell 3\PycharmProjects\Project\CGI-Process-Monitoring-302-303\static\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell 2\Desktop\faculdade\3 ano\TFC\CGI-Process-Monitoring-302-303\static\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{822DB8BE-8C89-42C6-BB28-C875240A96A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40DA966-63B0-423B-8355-0823F7C4D9EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -673,7 +673,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.8984375" bestFit="1" customWidth="1"/>
@@ -715,6 +715,9 @@
         <v>8</v>
       </c>
       <c r="E2" s="3"/>
+      <c r="G2">
+        <v>8206365164</v>
+      </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -730,6 +733,9 @@
         <v>12</v>
       </c>
       <c r="E3" s="3"/>
+      <c r="G3">
+        <v>1725612465</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -1036,16 +1042,6 @@
       </c>
       <c r="E21">
         <v>6211195490</v>
-      </c>
-    </row>
-    <row r="34" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H34">
-        <v>8206365164</v>
-      </c>
-    </row>
-    <row r="35" spans="8:8" x14ac:dyDescent="0.25">
-      <c r="H35">
-        <v>1725612465</v>
       </c>
     </row>
   </sheetData>

</xml_diff>